<commit_message>
style(BAOCAO-DCEXP-01): got van phong toan bo 15 slides theo chuan ky su PE (humanizer)
</commit_message>
<xml_diff>
--- a/bang-so-lieu/Bang_so_lieu_chi_tiet_IrisEXP_VN.xlsx
+++ b/bang-so-lieu/Bang_so_lieu_chi_tiet_IrisEXP_VN.xlsx
@@ -497,7 +497,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Nguồn dữ liệu: Hồ sơ kỹ thuật công đoạn Điều chỉnh / Bảo chứng thân máy (Biên bản 保証工程連携会 lần 2–17 đến ngày 15/10/2026, tài liệu DR4 &amp; bảng tính PE) - Đối chiếu chéo ngày 26/10/2026</t>
+          <t>Nguồn dữ liệu: Hồ sơ kỹ thuật công đoạn Điều chỉnh / Bảo chứng thân máy (Biên bản 保証工程連携会 lần 2-17 đến ngày 15/10/2026, tài liệu DR4 &amp; bảng tính PE) - Đối chiếu chéo ngày 26/10/2026</t>
         </is>
       </c>
     </row>
@@ -972,7 +972,7 @@
       </c>
       <c r="M10" s="4" t="inlineStr">
         <is>
-          <t>ĐÃ HỦY BỎ (見送り/廃止) — Thay thế bằng Đề án No.25 (Quét liên tục bằng DP)</t>
+          <t>ĐÃ HỦY BỎ (見送り/廃止) - Thay thế bằng Đề án No.25 (Quét liên tục bằng DP)</t>
         </is>
       </c>
       <c r="N10" s="4" t="inlineStr">
@@ -1042,7 +1042,7 @@
       </c>
       <c r="M11" s="4" t="inlineStr">
         <is>
-          <t>ĐÃ HỦY ROBOT (見送り) — Đã đạt mục tiêu xóa bước nhờ Đề án JP No.3 (削除確定) &amp; No.6</t>
+          <t>ĐÃ HỦY ROBOT (見送り) - Đã đạt mục tiêu xóa bước nhờ Đề án JP No.3 (削除確定) &amp; No.6</t>
         </is>
       </c>
       <c r="N11" s="4" t="inlineStr">
@@ -1100,7 +1100,7 @@
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>Đang báo giá (見積中) — Không dùng số 25.000 USD của No.23</t>
+          <t>Đang báo giá (見積中) - Không dùng số 25.000 USD của No.23</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
@@ -1110,12 +1110,12 @@
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>Đang thực nghiệm kiểm chứng độ chính xác giữa DP và ISU (連携会 lần 13–17)</t>
+          <t>Đang thực nghiệm kiểm chứng độ chính xác giữa DP và ISU (連携会 lần 13-17)</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>IrisEXP改善提案まとめ.xlsx (Row 39); IrisEXP報告.pptx (Slide 3); 連携会 第7回.txt; 第13回–17回.pptx</t>
+          <t>IrisEXP改善提案まとめ.xlsx (Row 39); IrisEXP報告.pptx (Slide 3); 連携会 第7回.txt; 第13回-17回.pptx</t>
         </is>
       </c>
     </row>
@@ -1147,7 +1147,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Sử dụng Microphone + phần mềm AI phân tích phổ âm thanh và Camera nhiệt. Phía JP ước tính chi phí 600 vạn JPY (~40.000 USD: 100 vạn JPY gá/mic + 500 vạn JPY AI). Chuyển sang đề tài nghiên cứu dài hạn 2026–2030.</t>
+          <t>Sử dụng Microphone + phần mềm AI phân tích phổ âm thanh và Camera nhiệt. Phía JP ước tính chi phí 600 vạn JPY (~40.000 USD: 100 vạn JPY gá/mic + 500 vạn JPY AI). Chuyển sang đề tài nghiên cứu dài hạn 2026-2030.</t>
         </is>
       </c>
       <c r="G13" s="2" t="n">
@@ -1155,7 +1155,7 @@
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>40 (Kỳ vọng dài hạn 2026–2030)</t>
+          <t>40 (Kỳ vọng dài hạn 2026-2030)</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
@@ -1170,17 +1170,17 @@
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>600 vạn JPY (~40.000 USD) [Dài hạn 2026–2030]</t>
+          <t>600 vạn JPY (~40.000 USD) [Dài hạn 2026-2030]</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>Nghiên cứu dài hạn 2026–2030 (Không xin duyệt trong đợt MP này)</t>
+          <t>Nghiên cứu dài hạn 2026-2030 (Không xin duyệt trong đợt MP này)</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>Hoãn áp dụng ngắn hạn -&gt; Chuyển vào lộ trình R&amp;D dài hạn 2026–2030 (連携会 第8回, DR議事録)</t>
+          <t>Hoãn áp dụng ngắn hạn -&gt; Chuyển vào lộ trình R&amp;D dài hạn 2026-2030 (連携会 第8回, DR議事録)</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr">
@@ -1230,7 +1230,7 @@
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>Giảm 177s~215s/máy (tương đương giảm ~1,8–2,2 người ở Takt 97s); xóa thao tác đo thủ công</t>
+          <t>Giảm 177s~215s/máy (tương đương giảm ~1,8-2,2 người ở Takt 97s); xóa thao tác đo thủ công</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
@@ -1390,7 +1390,7 @@
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>Đề án bổ sung tháng 9 — Đang chờ bộ phận Thiết kế JP xác nhận</t>
+          <t>Đề án bổ sung tháng 9 - Đang chờ bộ phận Thiết kế JP xác nhận</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr">
@@ -1528,7 +1528,7 @@
       </c>
       <c r="M18" s="2" t="inlineStr">
         <is>
-          <t>Đề án bổ sung tháng 9 — Đang chờ báo giá / xác nhận phương án</t>
+          <t>Đề án bổ sung tháng 9 - Đang chờ báo giá / xác nhận phương án</t>
         </is>
       </c>
       <c r="N18" s="2" t="inlineStr">
@@ -1600,7 +1600,7 @@
       </c>
       <c r="M19" s="2" t="inlineStr">
         <is>
-          <t>Đề án bổ sung tháng 9 — Đang chờ TK JP xác nhận (song song phương án gá nam châm No.21)</t>
+          <t>Đề án bổ sung tháng 9 - Đang chờ TK JP xác nhận (song song phương án gá nam châm No.21)</t>
         </is>
       </c>
       <c r="N19" s="2" t="inlineStr">
@@ -1670,7 +1670,7 @@
       </c>
       <c r="M20" s="2" t="inlineStr">
         <is>
-          <t>Đề án bổ sung tháng 9 — Đang thảo luận tại DR công đoạn (DR議事録 R15–16, R41–42)</t>
+          <t>Đề án bổ sung tháng 9 - Đang thảo luận tại DR công đoạn (DR議事録 R15-16, R41-42)</t>
         </is>
       </c>
       <c r="N20" s="2" t="inlineStr">
@@ -1745,7 +1745,7 @@
       </c>
       <c r="N21" s="2" t="inlineStr">
         <is>
-          <t>IrisEXP VN改善案LIST.xlsx (Row 19); IrisEXP改善提案まとめ.xlsx (Row 48); IrisEXP 工程 (更新中) 3.xlsx (R187–R231)</t>
+          <t>IrisEXP VN改善案LIST.xlsx (Row 19); IrisEXP改善提案まとめ.xlsx (Row 48); IrisEXP 工程 (更新中) 3.xlsx (R187-R231)</t>
         </is>
       </c>
     </row>
@@ -1808,7 +1808,7 @@
       </c>
       <c r="M22" s="2" t="inlineStr">
         <is>
-          <t>Đề án bổ sung tháng 9 — Đang chờ báo giá / xem xét khả thi</t>
+          <t>Đề án bổ sung tháng 9 - Đang chờ báo giá / xem xét khả thi</t>
         </is>
       </c>
       <c r="N22" s="2" t="inlineStr">
@@ -1915,7 +1915,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Thiết kế JP thay đổi góc vát Puli từ 5° lên 35° và đổi vật liệu sang Belt đàn hồi (弾性ベルト) để tự triệt tiêu độ lệch. Lưu ý: VN hiện vẫn phát sinh 1–2 máy NG/tháng nên chỉ xóa sau khi xác nhận linh kiện mới ổn định.</t>
+          <t>Thiết kế JP thay đổi góc vát Puli từ 5° lên 35° và đổi vật liệu sang Belt đàn hồi (弾性ベルト) để tự triệt tiêu độ lệch. Lưu ý: VN hiện vẫn phát sinh 1-2 máy NG/tháng nên chỉ xóa sau khi xác nhận linh kiện mới ổn định.</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -1950,7 +1950,7 @@
       </c>
       <c r="M24" s="2" t="inlineStr">
         <is>
-          <t>Chờ QA phê duyệt — JP đã xác nhận hiệu quả Puli 35° + Belt đàn hồi; VN tiếp tục thu thập dữ liệu</t>
+          <t>Chờ QA phê duyệt - JP đã xác nhận hiệu quả Puli 35° + Belt đàn hồi; VN tiếp tục thu thập dữ liệu</t>
         </is>
       </c>
       <c r="N24" s="2" t="inlineStr">
@@ -2067,7 +2067,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>PHẦN A: CHI TIẾT 25 HẠNG MỤC BOM CỦA ĐỀ ÁN NO.22 — TỰ ĐỘNG HÓA KIỂM TRA THÔNG MẠCH, TIẾP ĐỊA, CÁCH ĐIỆN CHỊU ÁP (ĐỀ NGHỊ PHÊ DUYỆT)</t>
+          <t>PHẦN A: CHI TIẾT 25 HẠNG MỤC BOM CỦA ĐỀ ÁN NO.22 - TỰ ĐỘNG HÓA KIỂM TRA THÔNG MẠCH, TIẾP ĐỊA, CÁCH ĐIỆN CHỊU ÁP (ĐỀ NGHỊ PHÊ DUYỆT)</t>
         </is>
       </c>
     </row>
@@ -2966,7 +2966,7 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>Khớp tuyệt đối tổng Sheet 導通・耐圧検査設備リスト (Row 28)</t>
+          <t>Khớp với tổng Sheet 導通・耐圧検査設備リスト (Row 28)</t>
         </is>
       </c>
     </row>
@@ -3012,7 +3012,7 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>Khớp Sheet 自動導通・耐圧検査 (Row 3–4)</t>
+          <t>Khớp Sheet 自動導通・耐圧検査 (Row 3-4)</t>
         </is>
       </c>
     </row>
@@ -3042,7 +3042,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>PHẦN B: BẢNG CẢNH BÁO PHƯƠNG ÁN ROBOT ĐÃ HỦY SAU DR4 (TUYỆT ĐỐI KHÔNG CỘNG VÀO KINH PHÍ XIN DUYỆT)</t>
+          <t>PHẦN B: BẢNG CẢNH BÁO PHƯƠNG ÁN ROBOT ĐÃ HỦY SAU DR4 (Không cộng vào kinh phí xin duyệt)</t>
         </is>
       </c>
     </row>
@@ -3081,7 +3081,7 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>ĐÃ HỦY — Thay bằng quét liên tục qua DP (No.25 - Đang báo giá)</t>
+          <t>ĐÃ HỦY - Thay bằng quét liên tục qua DP (No.25 - Đang báo giá)</t>
         </is>
       </c>
     </row>
@@ -3120,7 +3120,7 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>ĐÃ HỦY — Thay bằng đọc log U201 qua Host PC &amp; bảo chứng USB khi nạp FW</t>
+          <t>ĐÃ HỦY - Thay bằng đọc log U201 qua Host PC &amp; bảo chứng USB khi nạp FW</t>
         </is>
       </c>
     </row>
@@ -3153,7 +3153,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>BẢNG TỔNG HỢP ĐỐI CHIẾU CẢ 3 CỨ ĐIỂM: NHẬT BẢN (JP) – TRUNG QUỐC (CN) – VIỆT NAM (VN)</t>
+          <t>BẢNG TỔNG HỢP ĐỐI CHIẾU CẢ 3 CỨ ĐIỂM: NHẬT BẢN (JP) - TRUNG QUỐC (CN) - VIỆT NAM (VN)</t>
         </is>
       </c>
     </row>
@@ -3251,7 +3251,7 @@
       <c r="H5" t="inlineStr">
         <is>
           <t>• Hệ thống Mini PC (chuẩn Spica): ~40.000 JPY/bộ (1 bộ điều khiển 4 máy)
-• Dự toán phần mềm chuyển U413 sang lần bật máy đầu tiên: ~225–250 vạn JPY (tiết kiệm 42 vạn JPY/năm)
+• Dự toán phần mềm chuyển U413 sang lần bật máy đầu tiên: ~225-250 vạn JPY (tiết kiệm 42 vạn JPY/năm)
 • [Tham khảo dài hạn 2026-2030] AI âm thanh lạ: 600 vạn JPY (~40.000 USD)</t>
         </is>
       </c>
@@ -3262,7 +3262,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>IrisEXP改善提案まとめ.xlsx (No.1–7); IrisEXP 工程 (更新中) 3.xlsx; 2026年9月24日打ち合わせ資料.pptx; 第8回..第17回.pptx</t>
+          <t>IrisEXP改善提案まとめ.xlsx (No.1-7); IrisEXP 工程 (更新中) 3.xlsx; 2026年9月24日打ち合わせ資料.pptx; 第8回..第17回.pptx</t>
         </is>
       </c>
     </row>
@@ -3311,7 +3311,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>IrisEXP cn改善案list.xlsx; IrisEXP改善提案まとめ.xlsx (No.8–17, No.38); 第8回打ち合わせ資料.pptx (Slide 7)</t>
+          <t>IrisEXP cn改善案list.xlsx; IrisEXP改善提案まとめ.xlsx (No.8-17, No.38); 第8回打ち合わせ資料.pptx (Slide 7)</t>
         </is>
       </c>
     </row>
@@ -3334,13 +3334,13 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Sản lượng kế hoạch: 16.000 máy/tháng. Takt time giảm từ 114s (Iris2024) xuống 97s (IrisEXP). Tổng thời gian hiện tại: 2.350s/máy (39 bước, K1–K8), bố trí 14 người (hoặc 15 người theo slide DR4); nếu không cải tiến ở Takt 97s cần 18 người (17,62 người).</t>
+          <t>Sản lượng kế hoạch: 16.000 máy/tháng. Takt time giảm từ 114s (Iris2024) xuống 97s (IrisEXP). Tổng thời gian hiện tại: 2.350s/máy (39 bước, K1-K8), bố trí 14 người (hoặc 15 người theo slide DR4); nếu không cải tiến ở Takt 97s cần 18 người (17,62 người).</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
           <t>• Mục tiêu PDCA đến T3/2027: Giảm &gt;=50% = -1.175s/máy (xuống &lt;=1.175s/máy).
-• Tổng tiềm năng các đề án VN có định lượng (không trùng No.23): ~599,32s – 611,32s/máy (chưa gộp các mục đồng bộ JP/CN).
+• Tổng tiềm năng các đề án VN có định lượng (không trùng No.23): ~599,32s - 611,32s/máy (chưa gộp các mục đồng bộ JP/CN).
 • Thực tích PDCA đã đo đạc đến T10/2026: -4,32s/máy (0,18%).</t>
         </is>
       </c>
@@ -3363,7 +3363,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Iris EXPのVN提案.xlsx; IrisEXP VN改善案LIST.xlsx; IrisEXP改善提案まとめ.xlsx (No.18–37); DSLK Điều chỉnh Iris.xlsx; 調整工程計画.xlsx; KDTVN-A-QA-QA-BM-003-F (T5–T10)</t>
+          <t>Iris EXPのVN提案.xlsx; IrisEXP VN改善案LIST.xlsx; IrisEXP改善提案まとめ.xlsx (No.18-37); DSLK Điều chỉnh Iris.xlsx; 調整工程計画.xlsx; KDTVN-A-QA-QA-BM-003-F (T5-T10)</t>
         </is>
       </c>
     </row>
@@ -3392,7 +3392,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>BẢNG THEO DÕI LỘ TRÌNH PDCA HÀNG THÁNG (T4/2026 – T3/2027) VÀ SO SÁNH HIỆU QUẢ TRƯỚC / SAU (BEFORE / AFTER)</t>
+          <t>BẢNG THEO DÕI LỘ TRÌNH PDCA HÀNG THÁNG (T4/2026 - T3/2027) VÀ SO SÁNH HIỆU QUẢ TRƯỚC / SAU (BEFORE / AFTER)</t>
         </is>
       </c>
     </row>
@@ -3527,7 +3527,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Hoàn thành đo đạc hiện trạng 39 thao tác qua 8 trạm K1–K8: Tổng thời gian = 2.350 giây/máy (14 công nhân).</t>
+          <t>Hoàn thành đo đạc hiện trạng 39 thao tác qua 8 trạm K1-K8: Tổng thời gian = 2.350 giây/máy (14 công nhân).</t>
         </is>
       </c>
     </row>
@@ -3623,7 +3623,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Họp 連携会 lần 9–12, bổ sung 9 đề án VN (nâng lên 37 đề án độc lập, 38 đề án cả AI WeChat CN).</t>
+          <t>Họp 連携会 lần 9-12, bổ sung 9 đề án VN (nâng lên 37 đề án độc lập, 38 đề án cả AI WeChat CN).</t>
         </is>
       </c>
     </row>
@@ -3655,7 +3655,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Họp 連携会 lần 13–16; đã xóa 2 bước bấm đổi ngôn ngữ sang English (1,44s) và 2 bước kiểm tra cảnh báo Toner (2,88s) = giảm 4,32s. Tạm chưa đạt kế hoạch do JP chưa hoàn thành DR thiết kế công đoạn.</t>
+          <t>Họp 連携会 lần 13-16; đã xóa 2 bước bấm đổi ngôn ngữ sang English (1,44s) và 2 bước kiểm tra cảnh báo Toner (2,88s) = giảm 4,32s. Tạm chưa đạt kế hoạch do JP chưa hoàn thành DR thiết kế công đoạn.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Vietnam proposal prices and exact 25 BOM items from Iris EXPのVN提案.xlsx with humanizer
</commit_message>
<xml_diff>
--- a/bang-so-lieu/Bang_so_lieu_chi_tiet_IrisEXP_VN.xlsx
+++ b/bang-so-lieu/Bang_so_lieu_chi_tiet_IrisEXP_VN.xlsx
@@ -39,7 +39,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -54,11 +54,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00E2EFDA"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
   </fills>
@@ -88,7 +83,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -97,9 +92,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -865,17 +857,17 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>Tự động hóa kiểm tra thông mạch, tiếp địa, cách điện chịu áp (自動導通・耐圧検査の自動化)</t>
+          <t>Tự động hóa kiểm tra thông mạch, tiếp đất và chịu áp cách điện (導通・接地および絶縁耐圧を確認)</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>Công nhân cắm dây nguồn, kẹp que đo tiếp địa, bấm máy đo và chít barcode thủ công (20s tiếp địa + 10s chịu áp = 30s/máy).</t>
+          <t>Công nhân cắm dây nguồn, kẹp que đo tiếp đất, bấm máy đo cao áp và xác nhận thủ công (20s tiếp đất + 10s chịu áp = 30s/máy).</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>Chế tạo cụm Xylanh khí nén tự động cắm nguồn/chạm kim đo + PLC FX5U + Barcode cố định kết nối máy Chroma 19032. Lưu ý DR4: Phải đo khi ĐÃ ĐÓNG VỎ MÁY tại A-3 để phát hiện kẹt dây.</t>
+          <t>Chế tạo JIG kết nối + kiểm tra tự động (PLC Mitsubishi FX5U-64MT/ES, Module FX5-16EYR/ES, HMI Wecon PI3070ig, 6 Xylanh SMC MGCLB16/CXSL15, 5 Van SY5120, 2 Cảm biến quang E3Z-LS61, Khung nhôm Misumi LCF8-4040). Đo khi ĐÃ ĐÓNG VỎ MÁY theo DR4.</t>
         </is>
       </c>
       <c r="G9" s="3" t="n">
@@ -894,7 +886,7 @@
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
-          <t>3.911,15 USD (BOM) / 3.911,54 USD (101,7tr) / 4.000 USD (纏め)</t>
+          <t>3.911,15 USD (BOM 25 mục) / 3.911,54 USD (101,7tr) / 4.000 USD (纏め)</t>
         </is>
       </c>
       <c r="L9" s="3" t="inlineStr">
@@ -904,7 +896,7 @@
       </c>
       <c r="M9" s="3" t="inlineStr">
         <is>
-          <t>Phương án khả thi - Trình xin phê duyệt kinh phí đầu tư (cần chỉnh vị trí đo đóng vỏ theo DR4)</t>
+          <t>Đề nghị phê duyệt đầu tư (Triển khai ngay Đợt 1)</t>
         </is>
       </c>
       <c r="N9" s="3" t="inlineStr">
@@ -914,140 +906,134 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>No.23</t>
         </is>
       </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>Báo cáo T8 #6a / VN提案 #2 (ĐÃ HỦY)</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Báo cáo T8 #6a / VN提案 #2</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
         <is>
           <t>K4 -&gt; A-4</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t>[PHƯƠNG ÁN ĐÃ HỦY SAU DR4] Chế tạo Robot đặt bản thảo lên mặt kính ISU (ISU原稿セットロボット製作 - 廃止)</t>
-        </is>
-      </c>
-      <c r="E10" s="4" t="inlineStr">
-        <is>
-          <t>Công nhân mở nắp Platen, đặt/lấy từng tờ bản thảo lên mặt kính ISU: U411 (45s) + SITC-2 (35s) + Halftone (30s) = 110s/máy.</t>
-        </is>
-      </c>
-      <c r="F10" s="4" t="inlineStr">
-        <is>
-          <t>Dự kiến dùng cánh tay Robot (350tr) + mở rộng 2 cell băng tải (200tr) + cụm cấp nguồn (50tr) + định vị USB/LAN (50tr). ĐÃ QUYẾT ĐỊNH HỦY tại 連携会 lần 7 / DR4 vì chi phí quá lớn (650tr VNĐ), hoàn vốn &gt;6 năm, tốn diện tích.</t>
-        </is>
-      </c>
-      <c r="G10" s="4" t="n">
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Chế tạo Robot đặt bản thảo lên ISU, liên kết với Program để tự động điều chỉnh/kiểm tra (ISU U411 + SITC-2 + Halftone)</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>Công nhân mở nắp Platen, đặt/lấy từng tờ bản thảo lên mặt kính ISU: U411 (45s) + SITC-2 (35s) + Halftone máy màu (30s) = 110s/máy.</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>Dự toán tại Sheet 自動Scan tự động: (1) Bổ sung 2 Cell vào băng tải (200tr / $7.692,31) + (2) Bộ cấp nguồn máy in (50tr / $1.923,08) + (3) Bộ định vị kết nối dây USB/LAN (50tr / $1.923,08) + (4) Cánh tay Robot (350tr / $13.461,54). KTSX đã xác nhận giá TB; đồng thời tại DR4/連携会 đối chiếu với phương án bổ sung DP (No.25).</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="n">
         <v>110</v>
       </c>
-      <c r="H10" s="4" t="inlineStr">
-        <is>
-          <t>0 (Đã hủy, thay bằng No.25)</t>
-        </is>
-      </c>
-      <c r="I10" s="4" t="inlineStr">
-        <is>
-          <t>Tiết kiệm dự kiến 108.533.333 VNĐ/năm (4.174,36 USD/năm) không đủ bù chi phí 650tr VNĐ</t>
-        </is>
-      </c>
-      <c r="J10" s="4" t="n">
+      <c r="H10" s="3" t="n">
+        <v>110</v>
+      </c>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
+          <t>Giảm 110s/máy; tiết kiệm nhân công 108.533.333 VNĐ/năm (4.174,36 USD/năm)</t>
+        </is>
+      </c>
+      <c r="J10" s="3" t="n">
         <v>650000000</v>
       </c>
-      <c r="K10" s="4" t="inlineStr">
-        <is>
-          <t>25.000,00 USD (ĐÃ HỦY - KHÔNG DÙNG)</t>
-        </is>
-      </c>
-      <c r="L10" s="4" t="inlineStr">
-        <is>
-          <t>ĐÃ HỦY BỎ SAU DR4 (Tuyệt đối không đưa vào kinh phí xin duyệt)</t>
-        </is>
-      </c>
-      <c r="M10" s="4" t="inlineStr">
-        <is>
-          <t>ĐÃ HỦY BỎ (見送り/廃止) - Thay thế bằng Đề án No.25 (Quét liên tục bằng DP)</t>
-        </is>
-      </c>
-      <c r="N10" s="4" t="inlineStr">
+      <c r="K10" s="3" t="inlineStr">
+        <is>
+          <t>25.000,00 USD (Sheet 自動Scan tự động)</t>
+        </is>
+      </c>
+      <c r="L10" s="3" t="inlineStr">
+        <is>
+          <t>ĐÃ CÓ BÁO GIÁ TRONG VN提案.xlsx (Đối chiếu phương án thay bằng DP No.25 sau DR4)</t>
+        </is>
+      </c>
+      <c r="M10" s="3" t="inlineStr">
+        <is>
+          <t>Đã có dự toán 650tr VNĐ (25.000 USD); đang đối chiếu với phương án dùng DP (No.25)</t>
+        </is>
+      </c>
+      <c r="N10" s="3" t="inlineStr">
         <is>
           <t>Iris EXPのVN提案.xlsx (Sheets: 纏め, 自動Scan tự động); IrisEXP改善提案まとめ.xlsx (Row 37); 連携会 第7回.txt</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>No.24</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>Báo cáo T8 #7 / VN提案 #3 (ĐÃ HỦY)</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Báo cáo T8 #7 / VN提案 #3</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
         <is>
           <t>K4 -&gt; A-2/A-4</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>[PHƯƠNG ÁN ĐÃ HỦY SAU DR4] Tự động hóa kiểm tra nhận diện USB và tọa độ Panel U201 bằng Robot (USB認識・U201パネル座標検査ロボット - 廃止)</t>
-        </is>
-      </c>
-      <c r="E11" s="4" t="inlineStr">
-        <is>
-          <t>Công nhân cắm/rút USB kiểm tra nhận diện (15s) và dùng bút chạm 3 điểm trên màn hình U201 (15s) = 30s/máy.</t>
-        </is>
-      </c>
-      <c r="F11" s="4" t="inlineStr">
-        <is>
-          <t>Dự kiến làm cơ cấu tự động cắm USB và chạm màn hình (4.000 USD). ĐÃ HỦY vì hiệu quả đầu tư thấp; chuyển sang bảo chứng cổng USB qua bước nạp FW (JP No.6) và đọc log U201 từ Sub-Assy qua Host PC (JP No.3).</t>
-        </is>
-      </c>
-      <c r="G11" s="4" t="n">
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Robot kết nối USB, Camera đánh giá hiển thị Panel &amp; Camera AI cảm biến tọa độ, Robot chấm tọa độ U201 trên Panel</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Công nhân cắm/rút USB kiểm tra nhận biết (15s) và dùng bút chấm tọa độ U201 trên Panel (15s) = 30s/máy.</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>Dự toán tại Sheet 纏め Row 6-7: Chi phí thiết bị 4.000 USD (104.000.000 VNĐ), hiệu quả tương đương No.1 (-30s/máy). Phương án đối ứng không dùng Robot tại 連携会: bảo chứng cổng USB khi nạp FW (JP No.6) và đọc log U201 từ Sub-Assy qua Host PC (JP No.3).</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="n">
         <v>30</v>
       </c>
-      <c r="H11" s="4" t="inlineStr">
-        <is>
-          <t>30 (Nhờ xóa bước theo JP No.3 &amp; No.6, không tốn tiền Robot)</t>
-        </is>
-      </c>
-      <c r="I11" s="4" t="inlineStr">
-        <is>
-          <t>Xóa hoàn toàn 30s thao tác tay (trên 工程表 chuẩn giảm 15,12s U201 + 3,96s USB = 19,08s) mà không cần đầu tư Robot</t>
-        </is>
-      </c>
-      <c r="J11" s="4" t="inlineStr">
-        <is>
-          <t>Đã hủy (0 VNĐ)</t>
-        </is>
-      </c>
-      <c r="K11" s="4" t="inlineStr">
-        <is>
-          <t>4.000,00 USD (ĐÃ HỦY - KHÔNG DÙNG)</t>
-        </is>
-      </c>
-      <c r="L11" s="4" t="inlineStr">
-        <is>
-          <t>ĐÃ HỦY BỎ SAU DR4 (Chuyển sang giải pháp phần mềm 0 đồng TB)</t>
-        </is>
-      </c>
-      <c r="M11" s="4" t="inlineStr">
-        <is>
-          <t>ĐÃ HỦY ROBOT (見送り) - Đã đạt mục tiêu xóa bước nhờ Đề án JP No.3 (削除確定) &amp; No.6</t>
-        </is>
-      </c>
-      <c r="N11" s="4" t="inlineStr">
-        <is>
-          <t>Iris EXPのVN提案.xlsx (Sheet 纏め Row 6); IrisEXP改善提案まとめ.xlsx (Row 38); 連携会 第7回.txt</t>
+      <c r="H11" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>Giảm 30s/máy (No.1と同等の効果); tiết kiệm 29.600.000 VNĐ/năm (1.138,46 USD/năm)</t>
+        </is>
+      </c>
+      <c r="J11" s="3" t="n">
+        <v>104000000</v>
+      </c>
+      <c r="K11" s="3" t="inlineStr">
+        <is>
+          <t>4.000,00 USD (Sheet 纏め Row 6)</t>
+        </is>
+      </c>
+      <c r="L11" s="3" t="inlineStr">
+        <is>
+          <t>ĐÃ CÓ BÁO GIÁ TRONG VN提案.xlsx (Đối chiếu phương án phần mềm JP No.3 &amp; No.6)</t>
+        </is>
+      </c>
+      <c r="M11" s="3" t="inlineStr">
+        <is>
+          <t>Đã có dự toán 104tr VNĐ (4.000 USD); đối chiếu giải pháp phần mềm Host PC</t>
+        </is>
+      </c>
+      <c r="N11" s="3" t="inlineStr">
+        <is>
+          <t>Iris EXPのVN提案.xlsx (Sheet 纏め Row 6-7); IrisEXP改善提案まとめ.xlsx (Row 38); 連携会 第7回.txt</t>
         </is>
       </c>
     </row>
@@ -2036,7 +2022,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I38"/>
+  <dimension ref="A1:I46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2072,47 +2058,47 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>STT</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>Tên thiết bị / Linh kiện (Sheet 導通・耐圧検査設備リスト)</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>Quy cách / Model</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>Số lượng</t>
         </is>
       </c>
-      <c r="E5" s="5" t="inlineStr">
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>Đơn vị</t>
         </is>
       </c>
-      <c r="F5" s="5" t="inlineStr">
+      <c r="F5" s="4" t="inlineStr">
         <is>
           <t>Đơn giá (VNĐ)</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="G5" s="4" t="inlineStr">
         <is>
           <t>Thành tiền (VNĐ)</t>
         </is>
       </c>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="H5" s="4" t="inlineStr">
         <is>
           <t>Thành tiền (USD, tỷ giá 26.000)</t>
         </is>
       </c>
-      <c r="I5" s="5" t="inlineStr">
+      <c r="I5" s="4" t="inlineStr">
         <is>
           <t>Ghi chú trong nguồn</t>
         </is>
@@ -2124,32 +2110,36 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Nhôm định hình 30x30</t>
+          <t>PLC Mitsubishi FX5U-64MT/ES</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>30x30</t>
+          <t>FX5U-64MT/ES</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Thanh</t>
+          <t>Cái</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>290000</v>
+        <v>9500000</v>
       </c>
       <c r="G6" t="n">
-        <v>580000</v>
+        <v>9500000</v>
       </c>
       <c r="H6" t="n">
-        <v>22.31</v>
-      </c>
-      <c r="I6" t="inlineStr"/>
+        <v>365.38</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>codienhaiau.com</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -2157,32 +2147,36 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Nhôm định hình 30x60</t>
+          <t>Mạch Bảo Vệ CP30-BA (CP30-BA 2P 1-M 5A T)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>30x60</t>
+          <t>CP30-BA 2P 1-M 5A T</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Thanh</t>
+          <t>Cái</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>520000</v>
+        <v>650000</v>
       </c>
       <c r="G7" t="n">
-        <v>1560000</v>
+        <v>650000</v>
       </c>
       <c r="H7" t="n">
-        <v>60</v>
-      </c>
-      <c r="I7" t="inlineStr"/>
+        <v>25</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>vn.misumi-ec.com</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -2190,32 +2184,36 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Nhôm định hình 40x40</t>
+          <t>Module Mitsubishi FX5-16EYR/ES (16 Out Relay)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>40x40</t>
+          <t>FX5-16EYR/ES</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Thanh</t>
+          <t>Cái</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>450000</v>
+        <v>2000000</v>
       </c>
       <c r="G8" t="n">
-        <v>1800000</v>
+        <v>2000000</v>
       </c>
       <c r="H8" t="n">
-        <v>69.23</v>
-      </c>
-      <c r="I8" t="inlineStr"/>
+        <v>76.92</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>codienhaiau.com</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -2223,16 +2221,16 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Ke góc 30x30</t>
+          <t>Contactor Mitsubishi S-T32 32A 15kW AC200V 3P</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>30x30</t>
+          <t>S-T32 AC200V 3P</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>50</v>
+        <v>3</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -2240,15 +2238,19 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>6000</v>
+        <v>500000</v>
       </c>
       <c r="G9" t="n">
-        <v>300000</v>
+        <v>1500000</v>
       </c>
       <c r="H9" t="n">
-        <v>11.54</v>
-      </c>
-      <c r="I9" t="inlineStr"/>
+        <v>57.69</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>codienhaiau.com</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -2256,16 +2258,16 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Ke góc 40x40</t>
+          <t>Bộ nguồn Omron S8VK-C06024 2.5A 24VDC 60W</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>40x40</t>
+          <t>S8VK-C06024</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>50</v>
+        <v>1</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -2273,15 +2275,19 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>9000</v>
+        <v>700000</v>
       </c>
       <c r="G10" t="n">
-        <v>450000</v>
+        <v>700000</v>
       </c>
       <c r="H10" t="n">
-        <v>17.31</v>
-      </c>
-      <c r="I10" t="inlineStr"/>
+        <v>26.92</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>codienhaiau.com</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -2289,32 +2295,36 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Chân đế tăng chỉnh M12</t>
+          <t>Cầu đấu nguồn (BN30WPN50) gói 50pcs</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>M12</t>
+          <t>BN30WPN50</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Cái</t>
+          <t>Gói</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>35000</v>
+        <v>1000000</v>
       </c>
       <c r="G11" t="n">
-        <v>420000</v>
+        <v>1000000</v>
       </c>
       <c r="H11" t="n">
-        <v>16.15</v>
-      </c>
-      <c r="I11" t="inlineStr"/>
+        <v>38.46</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>vn.misumi-ec.com</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -2322,16 +2332,16 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Bánh xe có khóa</t>
+          <t>Chặn cầu đấu nguồn (BNE30W)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Có khóa</t>
+          <t>BNE30W</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -2339,15 +2349,19 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>85000</v>
+        <v>50000</v>
       </c>
       <c r="G12" t="n">
-        <v>680000</v>
+        <v>100000</v>
       </c>
       <c r="H12" t="n">
-        <v>26.15</v>
-      </c>
-      <c r="I12" t="inlineStr"/>
+        <v>3.85</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>vn.misumi-ec.com</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -2355,12 +2369,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Tấm Bakelit gia công đồ gá</t>
+          <t>Cầu đấu tín hiệu (BN10WPN50) gói 50 pcs</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Gia công theo bản vẽ</t>
+          <t>BN10WPN50</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -2368,19 +2382,23 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Bộ</t>
+          <t>Gói</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>5000000</v>
+        <v>700000</v>
       </c>
       <c r="G13" t="n">
-        <v>5000000</v>
+        <v>700000</v>
       </c>
       <c r="H13" t="n">
-        <v>192.31</v>
-      </c>
-      <c r="I13" t="inlineStr"/>
+        <v>26.92</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>vn.misumi-ec.com</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -2388,12 +2406,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Tấm Mica trong suốt che chắn an toàn</t>
+          <t>Chặn cầu đấu tín hiệu (BNE15W)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>T=5mm</t>
+          <t>BNE15W</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -2401,19 +2419,23 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Tấm</t>
+          <t>Cái</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>1400000</v>
+        <v>45000</v>
       </c>
       <c r="G14" t="n">
-        <v>2800000</v>
+        <v>90000</v>
       </c>
       <c r="H14" t="n">
-        <v>107.69</v>
-      </c>
-      <c r="I14" t="inlineStr"/>
+        <v>3.46</v>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>vn.misumi-ec.com</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -2421,12 +2443,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Đầu đọc Barcode cố định (Fixed Barcode Reader)</t>
+          <t>Jump nối cầu đấu tín hiệu (BNJ16FBPN10) (gói 10 pcs)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Đọc tự động S/N</t>
+          <t>BNJ16FBPN10</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -2434,19 +2456,23 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Cái</t>
+          <t>Gói</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>19000000</v>
+        <v>540000</v>
       </c>
       <c r="G15" t="n">
-        <v>19000000</v>
+        <v>540000</v>
       </c>
       <c r="H15" t="n">
-        <v>730.77</v>
-      </c>
-      <c r="I15" t="inlineStr"/>
+        <v>20.77</v>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>vn.misumi-ec.com</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -2454,32 +2480,36 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Xylanh khí nén SMC (Cắm nguồn / Chạm tiếp địa / Nhấn nút)</t>
+          <t>Chốt Chặn Thanh Ray (BNL6PN10) (gói 10 pcs)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>SMC</t>
+          <t>BNL6PN10</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Cái</t>
+          <t>Gói</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>2000000</v>
+        <v>110000</v>
       </c>
       <c r="G16" t="n">
-        <v>6000000</v>
+        <v>110000</v>
       </c>
       <c r="H16" t="n">
-        <v>230.77</v>
-      </c>
-      <c r="I16" t="inlineStr"/>
+        <v>4.23</v>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>vn.misumi-ec.com</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -2487,12 +2517,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Xylanh dẫn hướng SMC</t>
+          <t>Công tắc 2 vị trí ø30 TWN (ASN211N)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>SMC</t>
+          <t>ASN211N</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -2504,15 +2534,19 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>3500000</v>
+        <v>400000</v>
       </c>
       <c r="G17" t="n">
-        <v>3500000</v>
+        <v>400000</v>
       </c>
       <c r="H17" t="n">
-        <v>134.62</v>
-      </c>
-      <c r="I17" t="inlineStr"/>
+        <v>15.38</v>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>vn.misumi-ec.com</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -2520,16 +2554,16 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Van điện từ khí nén SMC (Solenoid Valve)</t>
+          <t>Còi báo FUJI DR30B6-EB</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>SMC</t>
+          <t>DR30B6-EB</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -2537,15 +2571,19 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>500000</v>
+        <v>300000</v>
       </c>
       <c r="G18" t="n">
-        <v>2000000</v>
+        <v>300000</v>
       </c>
       <c r="H18" t="n">
-        <v>76.92</v>
-      </c>
-      <c r="I18" t="inlineStr"/>
+        <v>11.54</v>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>baa.vn</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -2553,16 +2591,16 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Cảm biến hành trình Xylanh (Auto Switch)</t>
+          <t>Đèn tủ điện APN122DNPW</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>SMC</t>
+          <t>APN122DNPW</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -2570,15 +2608,19 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>150000</v>
+        <v>400000</v>
       </c>
       <c r="G19" t="n">
-        <v>1200000</v>
+        <v>400000</v>
       </c>
       <c r="H19" t="n">
-        <v>46.15</v>
-      </c>
-      <c r="I19" t="inlineStr"/>
+        <v>15.38</v>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>vn.misumi-ec.com</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -2586,32 +2628,36 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Giảm chấn thủy lực (Shock Absorber)</t>
+          <t>Máng nhựa 35x35 MRL3535 MORELE cây 2m</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>SMC</t>
+          <t>MRL3535</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Cái</t>
+          <t>Cây</t>
         </is>
       </c>
       <c r="F20" t="n">
-        <v>150000</v>
+        <v>50000</v>
       </c>
       <c r="G20" t="n">
-        <v>600000</v>
+        <v>100000</v>
       </c>
       <c r="H20" t="n">
-        <v>23.08</v>
-      </c>
-      <c r="I20" t="inlineStr"/>
+        <v>3.85</v>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>vanvh.com</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -2619,32 +2665,36 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Ống khí nén &amp; Đầu nối nhanh (Fitting)</t>
+          <t>Ray nhôm MRB-1000 gắn thiết bị trong tủ điện</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>SMC</t>
+          <t>MRB-1000</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Bộ</t>
+          <t>Thanh</t>
         </is>
       </c>
       <c r="F21" t="n">
         <v>200000</v>
       </c>
       <c r="G21" t="n">
-        <v>200000</v>
+        <v>400000</v>
       </c>
       <c r="H21" t="n">
-        <v>7.69</v>
-      </c>
-      <c r="I21" t="inlineStr"/>
+        <v>15.38</v>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>vn.misumi-ec.com</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -2652,12 +2702,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
+          <t>Tủ điện</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
           <t>Tủ điện điều khiển</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>500x400x200</t>
         </is>
       </c>
       <c r="D22" t="n">
@@ -2684,21 +2734,23 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="n">
-        <v>18</v>
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>18a</t>
+        </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>PLC Mitsubishi FX5U-32MT/ES</t>
+          <t>Van 1 chiều SY5120-5LZD-01</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>FX5U-32MT/ES</t>
+          <t>SY5120-5LZD-01</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -2706,28 +2758,34 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>13000000</v>
+        <v>1000000</v>
       </c>
       <c r="G23" t="n">
-        <v>13000000</v>
+        <v>5000000</v>
       </c>
       <c r="H23" t="n">
-        <v>500</v>
-      </c>
-      <c r="I23" t="inlineStr"/>
+        <v>192.31</v>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>sieuthidientudong.com</t>
+        </is>
+      </c>
     </row>
     <row r="24">
-      <c r="A24" t="n">
-        <v>19</v>
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>18b</t>
+        </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Màn hình cảm ứng HMI Mitsubishi GOT2000 (7 inch)</t>
+          <t>Xylanh MGCLB16-50</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>GT2107-WTBD</t>
+          <t>MGCLB16-50</t>
         </is>
       </c>
       <c r="D24" t="n">
@@ -2739,28 +2797,34 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>12000000</v>
+        <v>4000000</v>
       </c>
       <c r="G24" t="n">
-        <v>12000000</v>
+        <v>4000000</v>
       </c>
       <c r="H24" t="n">
-        <v>461.54</v>
-      </c>
-      <c r="I24" t="inlineStr"/>
+        <v>153.85</v>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>vn.misumi-ec.com</t>
+        </is>
+      </c>
     </row>
     <row r="25">
-      <c r="A25" t="n">
-        <v>20</v>
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>18c</t>
+        </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Bộ nguồn tổ ong 24VDC (Power Supply)</t>
+          <t>Xylanh CXSL15-50</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>24VDC</t>
+          <t>CXSL15-50</t>
         </is>
       </c>
       <c r="D25" t="n">
@@ -2772,32 +2836,38 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>650000</v>
+        <v>5100000</v>
       </c>
       <c r="G25" t="n">
-        <v>650000</v>
+        <v>5100000</v>
       </c>
       <c r="H25" t="n">
-        <v>25</v>
-      </c>
-      <c r="I25" t="inlineStr"/>
+        <v>196.15</v>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>vn.misumi-ec.com</t>
+        </is>
+      </c>
     </row>
     <row r="26">
-      <c r="A26" t="n">
-        <v>21</v>
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>18d</t>
+        </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Rơ-le trung gian (Relay 24VDC)</t>
+          <t>Xylanh CXSL15-70</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Omron MY2N</t>
+          <t>CXSL15-70</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -2805,65 +2875,73 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>95000</v>
+        <v>5600000</v>
       </c>
       <c r="G26" t="n">
-        <v>950000</v>
+        <v>5600000</v>
       </c>
       <c r="H26" t="n">
-        <v>36.54</v>
-      </c>
-      <c r="I26" t="inlineStr"/>
+        <v>215.38</v>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>vn.misumi-ec.com</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Nút nhấn Start / Stop / Emergency / Reset</t>
+          <t>Xylanh CXSL15-100</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Phi 22</t>
+          <t>CXSL15-100</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Bộ</t>
+          <t>Cái</t>
         </is>
       </c>
       <c r="F27" t="n">
-        <v>500000</v>
+        <v>6000000</v>
       </c>
       <c r="G27" t="n">
-        <v>500000</v>
+        <v>18000000</v>
       </c>
       <c r="H27" t="n">
-        <v>19.23</v>
-      </c>
-      <c r="I27" t="inlineStr"/>
+        <v>692.3099999999999</v>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>vn.misumi-ec.com</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Đèn tháp cảnh báo 3 màu có còi (Signal Tower)</t>
+          <t>Cảm biến quang E3Z-LS61</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>24VDC</t>
+          <t>E3Z-LS61</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -2874,25 +2952,29 @@
         <v>1500000</v>
       </c>
       <c r="G28" t="n">
-        <v>1500000</v>
+        <v>3000000</v>
       </c>
       <c r="H28" t="n">
-        <v>57.69</v>
-      </c>
-      <c r="I28" t="inlineStr"/>
+        <v>115.38</v>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>hoplongtech.com</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Dây điện, cầu đấu, máng cáp, vật tư phụ điện</t>
+          <t>Màn hình HMI Wecon PI3070ig</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Tổng hợp</t>
+          <t>PI3070ig</t>
         </is>
       </c>
       <c r="D29" t="n">
@@ -2900,126 +2982,172 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Bộ</t>
+          <t>Cái</t>
         </is>
       </c>
       <c r="F29" t="n">
-        <v>2000000</v>
+        <v>5000000</v>
       </c>
       <c r="G29" t="n">
-        <v>2000000</v>
+        <v>5000000</v>
       </c>
       <c r="H29" t="n">
-        <v>76.92</v>
-      </c>
-      <c r="I29" t="inlineStr"/>
+        <v>192.31</v>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>khangvietelectric.com</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
+        <v>22</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Thanh nhôm dựng khung LCF8-4040-2000</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>LCF8-4040-2000</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>15</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Thanh</t>
+        </is>
+      </c>
+      <c r="F30" t="n">
+        <v>500000</v>
+      </c>
+      <c r="G30" t="n">
+        <v>7500000</v>
+      </c>
+      <c r="H30" t="n">
+        <v>288.46</v>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Misumi economy</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>23</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Ke góc HBLTS8-45</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>HBLTS8-45</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>50</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Cái</t>
+        </is>
+      </c>
+      <c r="F31" t="n">
+        <v>60000</v>
+      </c>
+      <c r="G31" t="n">
+        <v>3000000</v>
+      </c>
+      <c r="H31" t="n">
+        <v>115.38</v>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Misumi</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>24</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Nut HNTP8-8</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>HNTP8-8</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>100</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Cái</t>
+        </is>
+      </c>
+      <c r="F32" t="n">
+        <v>20000</v>
+      </c>
+      <c r="G32" t="n">
+        <v>2000000</v>
+      </c>
+      <c r="H32" t="n">
+        <v>76.92</v>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Misumi</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
         <v>25</v>
       </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>Gia công chi tiết cơ khí chính xác (Đầu kẹp phích cắm, giá đỡ...)</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>Gia công CNC</t>
-        </is>
-      </c>
-      <c r="D30" t="n">
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Chi phí khác (bao gồm các chi tiết gia công và các thiết bị điện phát sinh)</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Gia công &amp; phụ kiện</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
         <v>1</v>
       </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>Bộ</t>
-        </is>
-      </c>
-      <c r="F30" t="n">
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Gói</t>
+        </is>
+      </c>
+      <c r="F33" t="n">
         <v>20000000</v>
       </c>
-      <c r="G30" t="n">
+      <c r="G33" t="n">
         <v>20000000</v>
       </c>
-      <c r="H30" t="n">
+      <c r="H33" t="n">
         <v>769.23</v>
       </c>
-      <c r="I30" t="inlineStr"/>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>TỔNG CỘNG BOM (25 MỤC)</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr"/>
-      <c r="C31" t="inlineStr"/>
-      <c r="D31" t="inlineStr"/>
-      <c r="E31" t="inlineStr"/>
-      <c r="F31" t="inlineStr"/>
-      <c r="G31" t="n">
-        <v>101690000</v>
-      </c>
-      <c r="H31" t="n">
-        <v>3911.15</v>
-      </c>
-      <c r="I31" t="inlineStr">
-        <is>
-          <t>Khớp với tổng Sheet 導通・耐圧検査設備リスト (Row 28)</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>TRONG ĐÓ: 24 MỤC ĐÃ CÓ GIÁ CỐ ĐỊNH (Trừ Mục 17 Tủ điện)</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr"/>
-      <c r="C32" t="inlineStr"/>
-      <c r="D32" t="inlineStr"/>
-      <c r="E32" t="inlineStr"/>
-      <c r="F32" t="inlineStr"/>
-      <c r="G32" t="n">
-        <v>96690000</v>
-      </c>
-      <c r="H32" t="n">
-        <v>3718.85</v>
-      </c>
-      <c r="I32" t="inlineStr">
-        <is>
-          <t>Nếu tách riêng Mục 17 (5.000.000 VNĐ) ghi "Xin báo giá"</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>SỐ LÀM TRÒN TRÊN SHEET THUYẾT MINH (自動導通・耐圧検査)</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr"/>
-      <c r="C33" t="inlineStr"/>
-      <c r="D33" t="inlineStr"/>
-      <c r="E33" t="inlineStr"/>
-      <c r="F33" t="inlineStr"/>
-      <c r="G33" t="n">
-        <v>101700000</v>
-      </c>
-      <c r="H33" t="n">
-        <v>3911.54</v>
-      </c>
-      <c r="I33" t="inlineStr">
-        <is>
-          <t>Khớp Sheet 自動導通・耐圧検査 (Row 3-4)</t>
-        </is>
-      </c>
+      <c r="I33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>SỐ LÀM TRÒN TRÊN SHEET TỔNG HỢP (纏め)</t>
+          <t>TỔNG CỘNG BOM ĐỀ ÁN 1 (No.22 - 25 MỤC)</t>
         </is>
       </c>
       <c r="B34" t="inlineStr"/>
@@ -3028,99 +3156,357 @@
       <c r="E34" t="inlineStr"/>
       <c r="F34" t="inlineStr"/>
       <c r="G34" t="n">
-        <v>104000000</v>
+        <v>101690000</v>
       </c>
       <c r="H34" t="n">
-        <v>4000</v>
+        <v>3911.15</v>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>Khớp Sheet 纏め (Row 2: 4,000 USD)</t>
+          <t>Khớp với tổng Sheet 導通・耐圧検査設備リスト (Row 31-32)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>TRONG ĐÓ: 24 MỤC ĐÃ CÓ GIÁ CỐ ĐỊNH (Trừ Mục 17 Tủ điện)</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr"/>
+      <c r="C35" t="inlineStr"/>
+      <c r="D35" t="inlineStr"/>
+      <c r="E35" t="inlineStr"/>
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" t="n">
+        <v>96690000</v>
+      </c>
+      <c r="H35" t="n">
+        <v>3718.85</v>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Nếu tách riêng Mục 17 (5.000.000 VNĐ) ghi "Xin báo giá"</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>PHẦN B: BẢNG CẢNH BÁO PHƯƠNG ÁN ROBOT ĐÃ HỦY SAU DR4 (Không cộng vào kinh phí xin duyệt)</t>
+          <t>SỐ LÀM TRÒN TRÊN SHEET THUYẾT MINH (自動導通・耐圧検査)</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr"/>
+      <c r="C36" t="inlineStr"/>
+      <c r="D36" t="inlineStr"/>
+      <c r="E36" t="inlineStr"/>
+      <c r="F36" t="inlineStr"/>
+      <c r="G36" t="n">
+        <v>101700000</v>
+      </c>
+      <c r="H36" t="n">
+        <v>3911.54</v>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Khớp Sheet 自動導通・耐圧検査 (Row 3-4)</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>No.23 (ĐÃ HỦY)</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>Mở rộng 2 cell băng tải (200tr) + Cấp nguồn (50tr) + Định vị USB/LAN (50tr) + Cánh tay Robot đặt bản thảo ISU (350tr)</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>Đã hủy tại 連携会 7 / DR4</t>
-        </is>
-      </c>
-      <c r="D37" t="n">
+          <t>SỐ LÀM TRÒN TRÊN SHEET TỔNG HỢP (纏め)</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr"/>
+      <c r="C37" t="inlineStr"/>
+      <c r="D37" t="inlineStr"/>
+      <c r="E37" t="inlineStr"/>
+      <c r="F37" t="inlineStr"/>
+      <c r="G37" t="n">
+        <v>104000000</v>
+      </c>
+      <c r="H37" t="n">
+        <v>4000</v>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Khớp Sheet 纏め (Row 2: 4,000 USD)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>PHẦN B: CHI TIẾT BÁO GIÁ ĐỀ ÁN 2 (NO.23 - ROBOT ĐẶT BẢN THẢO ISU) &amp; ĐỀ ÁN 3 (NO.24 - ROBOT USB/U201) TRONG IRIS EXPのVN提案.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>No.23 - Mục 1</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Bổ sung 2 Cell vào băng tải (コンベアにセルを2台追加)</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Sheet 自動Scan tự động R3</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
         <v>1</v>
       </c>
-      <c r="E37" t="inlineStr">
+      <c r="E40" t="inlineStr">
         <is>
           <t>Hệ thống</t>
         </is>
       </c>
-      <c r="F37" t="n">
+      <c r="F40" t="n">
+        <v>200000000</v>
+      </c>
+      <c r="G40" t="n">
+        <v>200000000</v>
+      </c>
+      <c r="H40" t="n">
+        <v>7692.31</v>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Giảm tổng cộng 110s/máy (U411: 45s, SITC-2: 35s, Halftone: 30s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>No.23 - Mục 2</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Bộ cấp nguồn cho máy in: bộ điều khiển + chi tiết cơ khí, gia công</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Sheet 自動Scan tự động R4</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>1</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Bộ</t>
+        </is>
+      </c>
+      <c r="F41" t="n">
+        <v>50000000</v>
+      </c>
+      <c r="G41" t="n">
+        <v>50000000</v>
+      </c>
+      <c r="H41" t="n">
+        <v>1923.08</v>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Tiết kiệm nhân công: 108.533.333 VNĐ/năm (4.174,36 USD/năm)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>No.23 - Mục 3</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Bộ định vị kết nối dây USB/ dây LAN (USB/LAN位置決め装置)</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Sheet 自動Scan tự động R5</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>1</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Bộ</t>
+        </is>
+      </c>
+      <c r="F42" t="n">
+        <v>50000000</v>
+      </c>
+      <c r="G42" t="n">
+        <v>50000000</v>
+      </c>
+      <c r="H42" t="n">
+        <v>1923.08</v>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Đối chiếu phương án thay bằng DP liên tục (No.25) tại DR4</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>No.23 - Mục 4</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Cánh tay Robot (ロボットアーム)</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Sheet 自動Scan tự động R6</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>1</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Bộ</t>
+        </is>
+      </c>
+      <c r="F43" t="n">
+        <v>350000000</v>
+      </c>
+      <c r="G43" t="n">
+        <v>350000000</v>
+      </c>
+      <c r="H43" t="n">
+        <v>13461.54</v>
+      </c>
+      <c r="I43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>CỘNG NO.23</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>TỔNG ĐỀ ÁN 2 (No.23 - Tự động hóa Scan bản thảo bằng Robot)</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Sheet 自動Scan tự động R7</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>1</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Hệ thống</t>
+        </is>
+      </c>
+      <c r="F44" t="n">
         <v>650000000</v>
       </c>
-      <c r="G37" t="n">
+      <c r="G44" t="n">
         <v>650000000</v>
       </c>
-      <c r="H37" t="n">
+      <c r="H44" t="n">
         <v>25000</v>
       </c>
-      <c r="I37" t="inlineStr">
-        <is>
-          <t>ĐÃ HỦY - Thay bằng quét liên tục qua DP (No.25 - Đang báo giá)</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>No.24 (ĐÃ HỦY)</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>Robot tự động cắm rút USB và chạm kiểm tra tọa độ Panel U201</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>Đã hủy tại 連携会 7 / DR4</t>
-        </is>
-      </c>
-      <c r="D38" t="n">
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Tiết kiệm 110s/máy = 108.533.333 VNĐ/năm (4.174,36 USD/năm)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>CỘNG NO.24</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>TỔNG ĐỀ ÁN 3 (No.24 - Robot kết nối USB, Camera đánh giá Panel &amp; Camera AI + Robot chấm tọa độ U201)</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Sheet 纏め R6-R7</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
         <v>1</v>
       </c>
-      <c r="E38" t="inlineStr">
+      <c r="E45" t="inlineStr">
         <is>
           <t>Hệ thống</t>
         </is>
       </c>
-      <c r="F38" t="n">
+      <c r="F45" t="n">
         <v>104000000</v>
       </c>
-      <c r="G38" t="n">
+      <c r="G45" t="n">
         <v>104000000</v>
       </c>
-      <c r="H38" t="n">
+      <c r="H45" t="n">
         <v>4000</v>
       </c>
-      <c r="I38" t="inlineStr">
-        <is>
-          <t>ĐÃ HỦY - Thay bằng đọc log U201 qua Host PC &amp; bảo chứng USB khi nạp FW</t>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>Giảm 30s/máy (15s USB + 15s U201), tiết kiệm 29.600.000 VNĐ/năm (1.138,46 USD/năm)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>TỔNG 3 ĐỀ ÁN</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>TỔNG CỘNG 3 ĐỀ ÁN CÓ BÁO GIÁ TRONG IRIS EXPのVN提案.xlsx (No.22 + No.23 + No.24)</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Theo BOM No.22 + No.23 + No.24</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>3</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Đề án</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr"/>
+      <c r="G46" t="n">
+        <v>855690000</v>
+      </c>
+      <c r="H46" t="n">
+        <v>32911.15</v>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>Theo thuyết minh: 855.700.000 VNĐ (32.911,54 USD) | Theo 纏め: 858.000.000 VNĐ (33.000 USD)</t>
         </is>
       </c>
     </row>
@@ -3165,52 +3551,52 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Cứ điểm</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Số đề án ban đầu (T8/2026)</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>Số đề án theo dõi PDCA (T9-T10)</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>Số đề án bản tổng hợp mới nhất</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>Hiện trạng thời gian / Nhân lực</t>
         </is>
       </c>
-      <c r="F4" s="5" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>Mục tiêu / Hiệu quả giảm thời gian</t>
         </is>
       </c>
-      <c r="G4" s="5" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>Hiệu quả nhân lực / Chi phí vận hành</t>
         </is>
       </c>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="H4" s="4" t="inlineStr">
         <is>
           <t>Kinh phí đầu tư đã có giá</t>
         </is>
       </c>
-      <c r="I4" s="5" t="inlineStr">
+      <c r="I4" s="4" t="inlineStr">
         <is>
           <t>Các hạng mục đang chờ báo giá (見積中)</t>
         </is>
       </c>
-      <c r="J4" s="5" t="inlineStr">
+      <c r="J4" s="4" t="inlineStr">
         <is>
           <t>Nguồn đối chiếu chính</t>
         </is>
@@ -3352,8 +3738,10 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>• Đề án No.22 (Tự động kiểm tra thông mạch, tiếp địa, chịu áp): 101.690.000 VNĐ (3.911,15 USD theo BOM 25 mục; hoặc 96.690.000 VNĐ nếu tách Mục 17 Tủ điện 5tr; thuyết minh ghi 101.700.000 VNĐ / 3.911,54 USD; 纏め ghi 4.000 USD).
-• [ĐÃ HỦY SAU DR4 - KHÔNG CỘNG]: Robot ISU No.23 (650tr VNĐ / 25.000 USD) &amp; Robot USB/U201 No.24 (4.000 USD).</t>
+          <t>• Đề án No.22 (Tự động kiểm tra thông mạch, tiếp đất, chịu áp): 101.690.000 VNĐ (3.911,15 USD theo BOM 25 mục; thuyết minh: 101.700.000 VNĐ / 3.911,54 USD; 纏め: 4.000 USD).
+• Đề án No.23 (Robot đặt bản thảo ISU): 650.000.000 VNĐ (25.000 USD).
+• Đề án No.24 (Robot USB/U201): 104.000.000 VNĐ (4.000 USD).
+=&gt; Tổng 3 đề án có báo giá trong Iris EXPのVN提案.xlsx: 855.690.000 VNĐ (32.911,15 USD; làm tròn trên 纏め là 33.000 USD / 858.000.000 VNĐ).</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -3404,32 +3792,32 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Tháng (FY2027)</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Mục tiêu giảm thời gian theo tháng (%)</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>Mục tiêu giảm thời gian (giây/máy)</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>Thực tích đã đo đạc (giây/máy)</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>Đánh giá (○/×/--)</t>
         </is>
       </c>
-      <c r="F4" s="5" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>Nội dung thực hiện thực tế (Do) trong biểu PDCA KDTVN-PE-③</t>
         </is>

</xml_diff>

<commit_message>
Replace 'công nhân' with 'người thao tác' across all slides and supporting data
</commit_message>
<xml_diff>
--- a/bang-so-lieu/Bang_so_lieu_chi_tiet_IrisEXP_VN.xlsx
+++ b/bang-so-lieu/Bang_so_lieu_chi_tiet_IrisEXP_VN.xlsx
@@ -588,12 +588,12 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Nạp FW qua USB từng máy, 1 công nhân đứng chờ rút/cắm USB (90s/máy).</t>
+          <t>Nạp FW qua USB từng máy, 1 người thao tác đứng chờ rút/cắm USB (90s/máy).</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>1 công nhân vận hành nạp đồng thời 4 máy qua mạng/Mini PC. Kết hợp phương án nạp sẵn FW tại Partner hoặc bỏ bước chờ nạp lại trên Line (chỉ kiểm tra version).</t>
+          <t>1 người thao tác vận hành nạp đồng thời 4 máy qua mạng/Mini PC. Kết hợp phương án nạp sẵn FW tại Partner hoặc bỏ bước chờ nạp lại trên Line (chỉ kiểm tra version).</t>
         </is>
       </c>
       <c r="G5" s="2" t="n">
@@ -726,7 +726,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Công nhân phải cắm/rút USB thủ công để chép file log kết quả kiểm tra (10s/máy).</t>
+          <t>Người thao tác phải cắm/rút USB thủ công để chép file log kết quả kiểm tra (10s/máy).</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -862,7 +862,7 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>Công nhân cắm dây nguồn, kẹp que đo tiếp đất, bấm máy đo cao áp và xác nhận thủ công (20s tiếp đất + 10s chịu áp = 30s/máy).</t>
+          <t>Người thao tác cắm dây nguồn, kẹp que đo tiếp đất, bấm máy đo cao áp và xác nhận thủ công (20s tiếp đất + 10s chịu áp = 30s/máy).</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
@@ -928,7 +928,7 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>Công nhân mở nắp Platen, đặt/lấy từng tờ bản thảo lên mặt kính ISU: U411 (45s) + SITC-2 (35s) + Halftone máy màu (30s) = 110s/máy.</t>
+          <t>Người thao tác mở nắp Platen, đặt/lấy từng tờ bản thảo lên mặt kính ISU: U411 (45s) + SITC-2 (35s) + Halftone máy màu (30s) = 110s/máy.</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
@@ -994,7 +994,7 @@
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>Công nhân cắm/rút USB kiểm tra nhận biết (15s) và dùng bút chấm tọa độ U201 trên Panel (15s) = 30s/máy.</t>
+          <t>Người thao tác cắm/rút USB kiểm tra nhận biết (15s) và dùng bút chấm tọa độ U201 trên Panel (15s) = 30s/máy.</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
@@ -1128,7 +1128,7 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Công nhân nghe bằng tai trong buồng cách âm (U030, U037, Fuser, FAN, Operation, MPF/DU = 40s/máy tại K6; ~90-120s tổng).</t>
+          <t>Người thao tác nghe bằng tai trong buồng cách âm (U030, U037, Fuser, FAN, Operation, MPF/DU = 40s/máy tại K6; ~90-120s tổng).</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -1268,7 +1268,7 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Công nhân cắm USB, quét barcode, bấm nút trên Panel và click xác nhận thủ công trên PC (130s/máy tại K8).</t>
+          <t>Người thao tác cắm USB, quét barcode, bấm nút trên Panel và click xác nhận thủ công trên PC (130s/máy tại K8).</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
@@ -1341,7 +1341,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Kiến nghị Thiết kế JP cải tiến mạch/phần mềm tự chẩn đoán trạng thái tiếp xúc mà không cần công nhân lắp/tháo đồ gá hộp mực.</t>
+          <t>Kiến nghị Thiết kế JP cải tiến mạch/phần mềm tự chẩn đoán trạng thái tiếp xúc mà không cần người thao tác lắp/tháo đồ gá hộp mực.</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -1478,7 +1478,7 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Công nhân phải bê đặt quả nặng đồ gá (2ND-6005/6006) vào khay giấy để kiểm tra độ đàn hồi đóng/mở Cassette 1, 2 (20s/máy), rất nặng và dễ rơi.</t>
+          <t>Người thao tác phải bê đặt quả nặng đồ gá (2ND-6005/6006) vào khay giấy để kiểm tra độ đàn hồi đóng/mở Cassette 1, 2 (20s/máy), rất nặng và dễ rơi.</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -1494,7 +1494,7 @@
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>Giảm 20s/máy, loại bỏ thao tác bê quả nặng gây mỏi tay công nhân</t>
+          <t>Giảm 20s/máy, loại bỏ thao tác bê quả nặng gây mỏi tay người thao tác</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
@@ -1618,7 +1618,7 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Công nhân tại công đoạn điều chỉnh K3 phải lắp và siết vít 6 cụm vỏ ngoài (90s/máy; trên 工程表 là 48,32s), làm gián đoạn luồng kiểm tra tự động.</t>
+          <t>Người thao tác tại công đoạn điều chỉnh K3 phải lắp và siết vít 6 cụm vỏ ngoài (90s/máy; trên 工程表 là 48,32s), làm gián đoạn luồng kiểm tra tự động.</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
@@ -1688,7 +1688,7 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Công nhân phải kéo khay, đổi cữ A5R/A6R/Folio/B4R/A3 và đặt đồ gá kiểm tra cảm biến lượng giấy 70%/30% nhiều lần (65s/máy tại K3; 66,68s trên 工程表).</t>
+          <t>Người thao tác phải kéo khay, đổi cữ A5R/A6R/Folio/B4R/A3 và đặt đồ gá kiểm tra cảm biến lượng giấy 70%/30% nhiều lần (65s/máy tại K3; 66,68s trên 工程表).</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
@@ -1758,7 +1758,7 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Công nhân phải lấy giấy và đặt thủ công vào Cassette 1/2 theo từng hướng xuất Centi/Inch (15s/máy tại K3).</t>
+          <t>Người thao tác phải lấy giấy và đặt thủ công vào Cassette 1/2 theo từng hướng xuất Centi/Inch (15s/máy tại K3).</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
@@ -1826,7 +1826,7 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Công nhân phải bật máy, mở/đóng nắp phải (COVER RIGHT) để kiểm tra công tắc nhận diện (25s/máy tại K4).</t>
+          <t>Người thao tác phải bật máy, mở/đóng nắp phải (COVER RIGHT) để kiểm tra công tắc nhận diện (25s/máy tại K4).</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
@@ -1896,7 +1896,7 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Sau khi Aging U950, công nhân phải cúi sát vào trong máy để đo độ lệch/khe hở Transfer Belt (5s tại K4 Thao tác chi tiết; 10,76s tại DSLK; 15,36s trên 工程表).</t>
+          <t>Sau khi Aging U950, người thao tác phải cúi sát vào trong máy để đo độ lệch/khe hở Transfer Belt (5s tại K4 Thao tác chi tiết; 10,76s tại DSLK; 15,36s trên 工程表).</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -1968,7 +1968,7 @@
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>Công nhân phải bấm nút đổi ngôn ngữ sang English (0,72s × 2 = 1,44s) và nhìn xác nhận cảnh báo trạng thái Toner xuất hiện rồi biến mất (1,44s × 2 = 2,88s).</t>
+          <t>Người thao tác phải bấm nút đổi ngôn ngữ sang English (0,72s × 2 = 1,44s) và nhìn xác nhận cảnh báo trạng thái Toner xuất hiện rồi biến mất (1,44s × 2 = 2,88s).</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
@@ -3915,7 +3915,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Hoàn thành đo đạc hiện trạng 39 thao tác qua 8 trạm K1-K8: Tổng thời gian = 2.350 giây/máy (14 công nhân).</t>
+          <t>Hoàn thành đo đạc hiện trạng 39 thao tác qua 8 trạm K1-K8: Tổng thời gian = 2.350 giây/máy (14 người thao tác).</t>
         </is>
       </c>
     </row>

</xml_diff>